<commit_message>
feat: add licensing workflow and release v1.1.0
</commit_message>
<xml_diff>
--- a/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
+++ b/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
@@ -797,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -809,7 +809,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Deployment Steps - copy the tool, update paths, install Python packages, and run</t>
+          <t>Deployment Steps - copy the tool, install dependencies, activate the license, and run</t>
         </is>
       </c>
       <c r="B1" s="21" t="n"/>
@@ -819,7 +819,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Recommended portable setup: keep Capacity_Optimizer_Control.xlsx inside 'Tooling Control Panel', then use Project_Root_Folder = '..', Input_Load_Folder = 'Data_Input', Input_Master_Folder = 'Data_Input', and Output_Folder = 'output'. 中文说明见右侧列。</t>
+          <t>Recommended portable setup: keep Capacity_Optimizer_Control.xlsx inside 'Tooling Control Panel', then use Project_Root_Folder = '..', Input_Load_Folder = 'Data_Input', Input_Master_Folder = 'Data_Input', Output_Folder = 'output', and place 'license.json' in the project root. 中文说明见右侧列。</t>
         </is>
       </c>
       <c r="B2" s="21" t="n"/>
@@ -922,17 +922,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Open the control workbook</t>
+          <t>Get the machine fingerprint</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Open 'Tooling Control Panel\Capacity_Optimizer_Control.xlsx'. Save the workbook after any edits, then go to the 'Control_Panel' sheet after reading this page.</t>
+          <t>If RSCP already gave you a trial/unbound license, skip to Step 6. Otherwise double-click 'get_machine_fingerprint.bat' in the project root. It creates 'machine_fingerprint.json' for this computer.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>打开 `Tooling Control Panel\Capacity_Optimizer_Control.xlsx`。每次修改后先保存，再切换到 `Control_Panel`。</t>
+          <t>如果 RSCP 已经直接给了试用版或 unbound 授权，可以跳到 Step 6。否则双击项目根目录里的 `get_machine_fingerprint.bat`，为当前电脑生成 `machine_fingerprint.json`。</t>
         </is>
       </c>
     </row>
@@ -944,17 +944,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Check migration settings</t>
+          <t>Request the license file</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>In Control_Panel, first check Project_Root_Folder, Input_Load_Folder, Input_Master_Folder, and Output_Folder. If the workbook stays in 'Tooling Control Panel', keep '..', 'Data_Input', 'Data_Input', and 'output'.</t>
+          <t>For a machine-locked license, send 'machine_fingerprint.json' to RSCP and request the signed 'license.json' for this computer. For a short-term trial, RSCP can issue an unbound license directly.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>先检查 `Project_Root_Folder`、`Input_Load_Folder`、`Input_Master_Folder`、`Output_Folder`。如果 workbook 仍然放在 `Tooling Control Panel` 目录中，默认保持 `.. / Data_Input / Data_Input / output` 即可。</t>
+          <t>如果要机绑授权，把 `machine_fingerprint.json` 发给 RSCP，并申请这台电脑专用的签名授权文件 `license.json`。如果只是短期试用，RSCP 也可以直接发 unbound 授权。</t>
         </is>
       </c>
     </row>
@@ -966,17 +966,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Check run settings</t>
+          <t>Place the license file</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Then review Scenario_Name, Start_Year, Start_Month_Num, Horizon_Months, Run_Mode, Verbose, and Skip_Validation_Errors.</t>
+          <t>Copy the signed 'license.json' into the project root, next to main.py and run_optimizer.bat.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>再检查运行参数，例如 `Scenario_Name`、起始年月、`Horizon_Months`、`Run_Mode`、`Verbose`、`Skip_Validation_Errors`。</t>
+          <t>把签名后的 `license.json` 放到项目根目录，也就是和 `main.py`、`run_optimizer.bat` 同级的位置。</t>
         </is>
       </c>
     </row>
@@ -988,17 +988,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Run the tool</t>
+          <t>Open the control workbook</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Press Ctrl+S to save first. Then click 'Run Optimizer' in Control_Panel, or run: python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx". If required packages are missing, the run batch file will stop and ask you to run setup_requirements.bat first.</t>
+          <t>Open 'Tooling Control Panel\Capacity_Optimizer_Control.xlsx'. Save the workbook after any edits, then go to the 'Control_Panel' sheet after reading this page.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>先按 `Ctrl+S` 保存，再在 `Control_Panel` 点击 `Run Optimizer`，或者在命令行运行：`python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"`。如果依赖没装好，运行批处理会先停止并提示你运行 `setup_requirements.bat`。</t>
+          <t>打开 `Tooling Control Panel\Capacity_Optimizer_Control.xlsx`。每次修改后先保存，再切换到 `Control_Panel`。</t>
         </is>
       </c>
     </row>
@@ -1010,17 +1010,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Review output</t>
+          <t>Check migration settings</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Open the 'output' folder and check the generated Excel reports. If Run_Mode = Both, the comparison workbook is also generated.</t>
+          <t>In Control_Panel, first check Project_Root_Folder, Input_Load_Folder, Input_Master_Folder, and Output_Folder. If the workbook stays in 'Tooling Control Panel', keep '..', 'Data_Input', 'Data_Input', and 'output'.</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>打开 `output` 文件夹查看结果。如果 `Run_Mode = Both`，还会额外生成一份 ModeA 和 ModeB 的对比报告。</t>
+          <t>先检查 `Project_Root_Folder`、`Input_Load_Folder`、`Input_Master_Folder`、`Output_Folder`。如果 workbook 仍然放在 `Tooling Control Panel` 目录中，默认保持 `.. / Data_Input / Data_Input / output` 即可。</t>
         </is>
       </c>
     </row>
@@ -1032,34 +1032,100 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
+          <t>Check run settings</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Then review Scenario_Name, Start_Year, Start_Month_Num, Horizon_Months, Run_Mode, Verbose, and Skip_Validation_Errors.</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>再检查运行参数，例如 `Scenario_Name`、起始年月、`Horizon_Months`、`Run_Mode`、`Verbose`、`Skip_Validation_Errors`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Step 10</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Run the tool</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Press Ctrl+S to save first. Then click 'Run Optimizer' in Control_Panel, or run: python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx". If required packages or license files are missing, the run batch file will stop and tell you what to do next.</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>先按 `Ctrl+S` 保存，再在 `Control_Panel` 点击 `Run Optimizer`，或者在命令行运行：`python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"`。如果依赖或授权文件缺失，运行批处理会先停止并明确告诉你下一步该做什么。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Step 11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Review output</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Open the 'output' folder and check the generated Excel reports. If Run_Mode = Both, the comparison workbook is also generated.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>打开 `output` 文件夹查看结果。如果 `Run_Mode = Both`，还会额外生成一份 ModeA 和 ModeB 的对比报告。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Step 12</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
           <t>If the run fails</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Check that the four migration settings point to valid folders, master_capacity.csv and planner files exist, and Python packages were installed successfully. If needed, run 'setup_requirements.bat' again.</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>如果运行失败，优先检查四个迁移路径是否正确，`master_capacity.csv` 和 planner 文件是否存在，以及依赖包是否安装成功。必要时重新运行 `setup_requirements.bat`。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Check that the four migration settings point to valid folders, master_capacity.csv and planner files exist, Python packages were installed successfully, and a valid 'license.json' is present in the project root. If needed, run 'setup_requirements.bat' again or regenerate 'machine_fingerprint.json'.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>如果运行失败，优先检查四个迁移路径是否正确，`master_capacity.csv` 和 planner 文件是否存在，依赖包是否安装成功，以及项目根目录里是否放了有效的 `license.json`。必要时重新运行 `setup_requirements.bat` 或重新生成 `machine_fingerprint.json`。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Where to continue: open the 'Control_Panel' sheet and start with the Migration Setup section.</t>
         </is>
       </c>
-      <c r="B16" s="21" t="n"/>
-      <c r="C16" s="21" t="n"/>
-      <c r="D16" s="22" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A19:D19"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1072,7 +1138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1091,158 +1157,224 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>1. Fill in the Control_Panel sheet.</t>
+          <t>1. Run setup_requirements.bat on a new computer.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>2. Planner and master data stay in CSV/Excel files on disk; the Python tool reads them directly.</t>
+          <t>2. For a short trial, ask RSCP for an unbound trial license and place license.json in the project root.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>3. Run: python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"</t>
+          <t>3. For a machine-locked license, run get_machine_fingerprint.bat and send machine_fingerprint.json to RSCP.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Or click the Run button inside Control_Panel.</t>
+          <t>4. Place the signed license.json in the project root.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>4. The tool writes one Excel result workbook per mode, with dashboard/report sheets included.</t>
+          <t>5. Fill in the Control_Panel sheet.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>6. Planner and master data stay in CSV/Excel files on disk; the Python tool reads them directly.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>KEY SETTINGS</t>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>7. Run: python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Project_Root_Folder: main project folder. Keep '..' when the workbook stays inside Tooling Control Panel.</t>
+          <t xml:space="preserve">   Or click the Run button inside Control_Panel.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Input_Load_Folder: planner folder name or path. Relative values are resolved from Project_Root_Folder.</t>
+          <t>8. The tool writes one Excel result workbook per mode, with dashboard/report sheets included.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Input_Master_Folder: master-data folder name or path. Relative values are resolved from Project_Root_Folder.</t>
-        </is>
-      </c>
+      <c r="A12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Output_Folder: output folder name or path. Relative values are resolved from Project_Root_Folder.</t>
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>KEY SETTINGS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Output_FileName: base output file name; mode and timestamp are appended automatically.</t>
+          <t>Project_Root_Folder: main project folder. Keep '..' when the workbook stays inside Tooling Control Panel.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Scenario_Name: planner scenario to load. If your input folder changes, type the scenario manually if needed.</t>
+          <t>Input_Load_Folder: planner folder name or path. Relative values are resolved from Project_Root_Folder.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Start_Year / Start_Month_Num: first planning bucket.</t>
+          <t>Input_Master_Folder: master-data folder name or path. Relative values are resolved from Project_Root_Folder.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Horizon_Months: number of months to optimize.</t>
+          <t>Output_Folder: output folder name or path. Relative values are resolved from Project_Root_Folder.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Run_Mode: ModeA, ModeB, or Both.</t>
+          <t>Output_FileName: base output file name; mode and timestamp are appended automatically.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Direct_Mode: keep 'Yes' for the folder-based CSV workflow.</t>
+          <t>Scenario_Name: planner scenario to load. If your input folder changes, type the scenario manually if needed.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Verbose: prints solver detail in the command window.</t>
+          <t>Start_Year / Start_Month_Num: first planning bucket.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Skip_Validation_Errors: only use 'Yes' when you intentionally want a forced run.</t>
+          <t>Horizon_Months: number of months to optimize.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr"/>
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Run_Mode: ModeA, ModeB, or Both.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>RESULT WORKBOOK CONTENT</t>
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Direct_Mode: keep 'Yes' for the folder-based CSV workflow.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Dashboard, Monthly_Trend, Bottleneck, WC_Heatmap, Product_Risk</t>
+          <t>Verbose: prints solver detail in the command window.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
+          <t>Skip_Validation_Errors: only use 'Yes' when you intentionally want a forced run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>LICENSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>license.json: required in the project root before the optimizer can run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Trial / unbound license: no machine fingerprint required; RSCP can issue it directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>get_machine_fingerprint.bat: creates machine_fingerprint.json for RSCP to issue a machine-locked license.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Run_Info: each output workbook records license status, license ID, customer, expiry date, and binding mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>RESULT WORKBOOK CONTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Monthly_Trend, Bottleneck, WC_Heatmap, Product_Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
           <t>Allocation_Detail, Allocation_Summary, Outsource_Summary, Unmet_Summary, WC_Load_Pct</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Binary_Feasibility, Validation_Issues, Run_Info</t>
         </is>
@@ -1259,7 +1391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C179"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1296,7 +1428,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Recommended portable setup: keep Project_Root_Folder = '..', Input folders = 'Data_Input', and Output_Folder = 'output'. See 'Deployment_Steps' for the full setup checklist.</t>
+          <t>Recommended portable setup: keep Project_Root_Folder = '..', Input folders = 'Data_Input', Output_Folder = 'output', and place 'license.json' in the project root. See 'Deployment_Steps' for the full setup checklist.</t>
         </is>
       </c>
       <c r="B3" s="21" t="n"/>
@@ -1310,7 +1442,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>C:\Users\super\capacity_optimizer</t>
+          <t>..</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -1555,7 +1687,7 @@
           <t>Run_Timestamp</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n"/>
+      <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="inlineStr">
         <is>
           <t>Filled by Python at runtime</t>
@@ -1568,7 +1700,7 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="16" t="n"/>
+      <c r="B20" s="16" t="inlineStr"/>
       <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Free text</t>
@@ -1610,7 +1742,7 @@
     <row r="27" ht="22" customHeight="1">
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Run Optimizer</t>
+          <t>Get Machine Fingerprint</t>
         </is>
       </c>
       <c r="C27" s="23" t="n"/>
@@ -1623,7 +1755,7 @@
     <row r="30" ht="22" customHeight="1">
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Open Output Folder</t>
+          <t>Run Optimizer</t>
         </is>
       </c>
       <c r="C30" s="23" t="n"/>
@@ -1633,166 +1765,34 @@
       <c r="C31" s="25" t="n"/>
     </row>
     <row r="32"/>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Open Output Folder</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="25" t="n"/>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Button note</t>
         </is>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Run Setup Dependencies once on a new computer. Save the workbook first (Ctrl+S) before clicking Run Optimizer. If dependencies are missing, Run Optimizer will stop and remind you.</t>
         </is>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="B33:C34"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="B24:C25"/>
@@ -1824,6 +1824,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: reorganize delivery workflow and release v1.1.1
</commit_message>
<xml_diff>
--- a/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
+++ b/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
@@ -121,7 +121,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -143,95 +143,11 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0B0B0"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B0B0B0"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -285,11 +201,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -812,19 +723,13 @@
           <t>Deployment Steps - copy the tool, install dependencies, activate the license, and run</t>
         </is>
       </c>
-      <c r="B1" s="21" t="n"/>
-      <c r="C1" s="21" t="n"/>
-      <c r="D1" s="22" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Recommended portable setup: keep Capacity_Optimizer_Control.xlsx inside 'Tooling Control Panel', then use Project_Root_Folder = '..', Input_Load_Folder = 'Data_Input', Input_Master_Folder = 'Data_Input', Output_Folder = 'output', and place 'license.json' in the project root. 中文说明见右侧列。</t>
-        </is>
-      </c>
-      <c r="B2" s="21" t="n"/>
-      <c r="C2" s="21" t="n"/>
-      <c r="D2" s="22" t="n"/>
+          <t>Recommended portable setup: keep Capacity_Optimizer_Control.xlsx inside 'Tooling Control Panel', then use Project_Root_Folder = '..', Input_Load_Folder = 'Data_Input', Input_Master_Folder = 'Data_Input', Output_Folder = 'output', and place 'license.json' in 'licenses\active\'. 中文说明见右侧列。</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -905,12 +810,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Double-click 'setup_requirements.bat' in the project root to install the required Python packages automatically.</t>
+          <t>Double-click 'runtime\setup_requirements.bat' to install the required Python packages automatically.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>双击项目根目录里的 `setup_requirements.bat`，自动安装所需 Python 依赖。</t>
+          <t>双击 `runtime\setup_requirements.bat`，自动安装所需 Python 依赖。</t>
         </is>
       </c>
     </row>
@@ -927,12 +832,12 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>If RSCP already gave you a trial/unbound license, skip to Step 6. Otherwise double-click 'get_machine_fingerprint.bat' in the project root. It creates 'machine_fingerprint.json' for this computer.</t>
+          <t>If RSCP already gave you a trial/unbound license, skip to Step 6. Otherwise double-click 'runtime\get_machine_fingerprint.bat'. It creates a timestamped fingerprint file under 'licenses\requests\'.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>如果 RSCP 已经直接给了试用版或 unbound 授权，可以跳到 Step 6。否则双击项目根目录里的 `get_machine_fingerprint.bat`，为当前电脑生成 `machine_fingerprint.json`。</t>
+          <t>如果 RSCP 已经直接给了试用版或 unbound 授权，可以跳到 Step 6。否则双击 `runtime\get_machine_fingerprint.bat`，它会在 `licenses\requests\` 下生成带时间戳的机器指纹文件。</t>
         </is>
       </c>
     </row>
@@ -949,12 +854,12 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>For a machine-locked license, send 'machine_fingerprint.json' to RSCP and request the signed 'license.json' for this computer. For a short-term trial, RSCP can issue an unbound license directly.</t>
+          <t>For a machine-locked license, send the fingerprint file from 'licenses\requests\' to RSCP and request the signed 'license.json' for this computer. For a short-term trial, RSCP can issue an unbound license directly.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>如果要机绑授权，把 `machine_fingerprint.json` 发给 RSCP，并申请这台电脑专用的签名授权文件 `license.json`。如果只是短期试用，RSCP 也可以直接发 unbound 授权。</t>
+          <t>如果要机绑授权，把 `licenses\requests\` 下生成的机器指纹文件发给 RSCP，并申请这台电脑专用的签名授权文件 `license.json`。如果只是短期试用，RSCP 也可以直接发 unbound 授权。</t>
         </is>
       </c>
     </row>
@@ -971,12 +876,12 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Copy the signed 'license.json' into the project root, next to main.py and run_optimizer.bat.</t>
+          <t>Copy the signed 'license.json' into 'licenses\active\license.json'. The legacy project-root 'license.json' path is still supported.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>把签名后的 `license.json` 放到项目根目录，也就是和 `main.py`、`run_optimizer.bat` 同级的位置。</t>
+          <t>把签名后的 `license.json` 放到 `licenses\active\license.json`。旧的项目根目录 `license.json` 方式仍然兼容。</t>
         </is>
       </c>
     </row>
@@ -1059,12 +964,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Press Ctrl+S to save first. Then click 'Run Optimizer' in Control_Panel, or run: python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx". If required packages or license files are missing, the run batch file will stop and tell you what to do next.</t>
+          <t>Press Ctrl+S to save first. Then click 'Run Optimizer' in Control_Panel, or run: python -m app.main --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx". If required packages or license files are missing, the run batch file will stop and tell you what to do next.</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>先按 `Ctrl+S` 保存，再在 `Control_Panel` 点击 `Run Optimizer`，或者在命令行运行：`python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"`。如果依赖或授权文件缺失，运行批处理会先停止并明确告诉你下一步该做什么。</t>
+          <t>先按 `Ctrl+S` 保存，再在 `Control_Panel` 点击 `Run Optimizer`，或者在命令行运行：`python -m app.main --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"`。如果依赖或授权文件缺失，运行批处理会先停止并明确告诉你下一步该做什么。</t>
         </is>
       </c>
     </row>
@@ -1103,12 +1008,12 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Check that the four migration settings point to valid folders, master_capacity.csv and planner files exist, Python packages were installed successfully, and a valid 'license.json' is present in the project root. If needed, run 'setup_requirements.bat' again or regenerate 'machine_fingerprint.json'.</t>
+          <t>Check that the four migration settings point to valid folders, master_capacity.csv and planner files exist, Python packages were installed successfully, and a valid license is present under 'licenses\active\license.json' or the legacy project-root path. If needed, run 'runtime\setup_requirements.bat' again or regenerate the machine fingerprint.</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>如果运行失败，优先检查四个迁移路径是否正确，`master_capacity.csv` 和 planner 文件是否存在，依赖包是否安装成功，以及项目根目录里是否放了有效的 `license.json`。必要时重新运行 `setup_requirements.bat` 或重新生成 `machine_fingerprint.json`。</t>
+          <t>如果运行失败，优先检查四个迁移路径是否正确，`master_capacity.csv` 和 planner 文件是否存在，依赖包是否安装成功，以及 `licenses\active\license.json` 或旧项目根目录下是否有有效授权。必要时重新运行 `runtime\setup_requirements.bat` 或重新生成机器指纹。</t>
         </is>
       </c>
     </row>
@@ -1118,9 +1023,6 @@
           <t>Where to continue: open the 'Control_Panel' sheet and start with the Migration Setup section.</t>
         </is>
       </c>
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1157,28 +1059,28 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>1. Run setup_requirements.bat on a new computer.</t>
+          <t>1. Run runtime\setup_requirements.bat on a new computer.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>2. For a short trial, ask RSCP for an unbound trial license and place license.json in the project root.</t>
+          <t>2. For a short trial, ask RSCP for an unbound trial license and place it in licenses\active\license.json.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>3. For a machine-locked license, run get_machine_fingerprint.bat and send machine_fingerprint.json to RSCP.</t>
+          <t>3. For a machine-locked license, run runtime\get_machine_fingerprint.bat and send the file from licenses\requests\ to RSCP.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>4. Place the signed license.json in the project root.</t>
+          <t>4. Place the signed license.json in licenses\active\license.json.</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1101,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>7. Run: python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"</t>
+          <t>7. Run: python -m app.main --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1226,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>license.json: required in the project root before the optimizer can run.</t>
+          <t>license.json: recommended location is licenses\active\license.json; the legacy project-root path is also supported.</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1240,7 @@
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>get_machine_fingerprint.bat: creates machine_fingerprint.json for RSCP to issue a machine-locked license.</t>
+          <t>runtime\get_machine_fingerprint.bat: creates a timestamped fingerprint file under licenses\requests\ for RSCP to issue a machine-locked license.</t>
         </is>
       </c>
     </row>
@@ -1422,17 +1324,13 @@
           <t>Migration Setup - update these cells first after copying the tool to another computer</t>
         </is>
       </c>
-      <c r="B2" s="21" t="n"/>
-      <c r="C2" s="22" t="n"/>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Recommended portable setup: keep Project_Root_Folder = '..', Input folders = 'Data_Input', Output_Folder = 'output', and place 'license.json' in the project root. See 'Deployment_Steps' for the full setup checklist.</t>
-        </is>
-      </c>
-      <c r="B3" s="21" t="n"/>
-      <c r="C3" s="22" t="n"/>
+          <t>Recommended portable setup: keep Project_Root_Folder = '..', Input folders = 'Data_Input', Output_Folder = 'output', and place 'license.json' in 'licenses\active\'. See 'Deployment_Steps' for the full setup checklist.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -1508,8 +1406,6 @@
           <t>Run Settings</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="22" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
@@ -1707,7 +1603,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
         <is>
@@ -1716,11 +1611,10 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>python main.py --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+          <t>python -m app.main --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"</t>
+        </is>
+      </c>
+    </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="18" t="inlineStr">
         <is>
@@ -1732,52 +1626,48 @@
           <t>Setup Dependencies</t>
         </is>
       </c>
-      <c r="C24" s="23" t="n"/>
+      <c r="C24" s="20" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="24" t="n"/>
-      <c r="C25" s="25" t="n"/>
-    </row>
-    <row r="26"/>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+    </row>
     <row r="27" ht="22" customHeight="1">
       <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Get Machine Fingerprint</t>
         </is>
       </c>
-      <c r="C27" s="23" t="n"/>
+      <c r="C27" s="20" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="24" t="n"/>
-      <c r="C28" s="25" t="n"/>
-    </row>
-    <row r="29"/>
+      <c r="B28" s="20" t="n"/>
+      <c r="C28" s="20" t="n"/>
+    </row>
     <row r="30" ht="22" customHeight="1">
       <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Run Optimizer</t>
         </is>
       </c>
-      <c r="C30" s="23" t="n"/>
+      <c r="C30" s="20" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="24" t="n"/>
-      <c r="C31" s="25" t="n"/>
-    </row>
-    <row r="32"/>
+      <c r="B31" s="20" t="n"/>
+      <c r="C31" s="20" t="n"/>
+    </row>
     <row r="33" ht="22" customHeight="1">
       <c r="B33" s="11" t="inlineStr">
         <is>
           <t>Open Output Folder</t>
         </is>
       </c>
-      <c r="C33" s="23" t="n"/>
+      <c r="C33" s="20" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="24" t="n"/>
-      <c r="C34" s="25" t="n"/>
-    </row>
-    <row r="35"/>
+      <c r="B34" s="20" t="n"/>
+      <c r="C34" s="20" t="n"/>
+    </row>
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
         <is>
@@ -1786,7 +1676,7 @@
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>Run Setup Dependencies once on a new computer. Save the workbook first (Ctrl+S) before clicking Run Optimizer. If dependencies are missing, Run Optimizer will stop and remind you.</t>
+          <t>On a new computer, click Setup Dependencies first. If RSCP gave you a trial/unbound license, place license.json in licenses\active and continue. Otherwise click Get Machine Fingerprint, send the generated file from licenses\requests to RSCP, place the returned license.json in licenses\active, save the workbook (Ctrl+S), and click Run Optimizer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add dashboard workcenter filters and license sheet
</commit_message>
<xml_diff>
--- a/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
+++ b/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Lists" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="Deployment_Steps" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Control_Panel" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="License" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Control_Panel" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -121,7 +122,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -143,11 +144,95 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -201,6 +286,20 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -723,6 +822,9 @@
           <t>Deployment Steps - copy the tool, install dependencies, activate the license, and run</t>
         </is>
       </c>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="22" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -730,6 +832,9 @@
           <t>Recommended portable setup: keep Capacity_Optimizer_Control.xlsx inside 'Tooling Control Panel', then use Project_Root_Folder = '..', Input_Load_Folder = 'Data_Input', Input_Master_Folder = 'Data_Input', Output_Folder = 'output', and place 'license.json' in 'licenses\active\'. 中文说明见右侧列。</t>
         </is>
       </c>
+      <c r="B2" s="21" t="n"/>
+      <c r="C2" s="21" t="n"/>
+      <c r="D2" s="22" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1023,6 +1128,9 @@
           <t>Where to continue: open the 'Control_Panel' sheet and start with the Migration Setup section.</t>
         </is>
       </c>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1293,6 +1401,264 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Current License</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>This sheet shows the currently detected license for this tool copy. Values refresh when the workbook is generated and again when the optimizer can save updates back to this file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>License_Status</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>Current validation status of the active license</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>License_Name</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>LIC-DEV-2026-0001</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>Current license ID / license name</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>License_Mode</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Internal / Machine Locked</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Friendly label such as Trial / Unbound or Commercial / Machine Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>License_Type</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>License type from license.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>Binding_Mode</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>machine_locked</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>Whether the license is unbound or machine locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Licensed_To</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>RSCP</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>Customer name recorded in the license</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Issue_Date</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>License issue date</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Expiry_Date</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>2027-12-31</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>License expiry date</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Machine_Name</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>HYC</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>Licensed machine label when applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>License_File_Path</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>C:\Users\super\capacity_optimizer\licenses\active\license.json</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>Detected license.json location</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Local development license</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>Note stored inside the license file</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>License validated successfully.</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>Last license inspection message</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1324,6 +1690,8 @@
           <t>Migration Setup - update these cells first after copying the tool to another computer</t>
         </is>
       </c>
+      <c r="B2" s="21" t="n"/>
+      <c r="C2" s="22" t="n"/>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -1331,6 +1699,8 @@
           <t>Recommended portable setup: keep Project_Root_Folder = '..', Input folders = 'Data_Input', Output_Folder = 'output', and place 'license.json' in 'licenses\active\'. See 'Deployment_Steps' for the full setup checklist.</t>
         </is>
       </c>
+      <c r="B3" s="21" t="n"/>
+      <c r="C3" s="22" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -1406,6 +1776,8 @@
           <t>Run Settings</t>
         </is>
       </c>
+      <c r="B8" s="21" t="n"/>
+      <c r="C8" s="22" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
@@ -1626,11 +1998,11 @@
           <t>Setup Dependencies</t>
         </is>
       </c>
-      <c r="C24" s="20" t="n"/>
+      <c r="C24" s="26" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="20" t="n"/>
+      <c r="B25" s="27" t="n"/>
+      <c r="C25" s="28" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="B27" s="11" t="inlineStr">
@@ -1638,11 +2010,11 @@
           <t>Get Machine Fingerprint</t>
         </is>
       </c>
-      <c r="C27" s="20" t="n"/>
+      <c r="C27" s="26" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="20" t="n"/>
-      <c r="C28" s="20" t="n"/>
+      <c r="B28" s="27" t="n"/>
+      <c r="C28" s="28" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="B30" s="11" t="inlineStr">
@@ -1650,11 +2022,11 @@
           <t>Run Optimizer</t>
         </is>
       </c>
-      <c r="C30" s="20" t="n"/>
+      <c r="C30" s="26" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="20" t="n"/>
-      <c r="C31" s="20" t="n"/>
+      <c r="B31" s="27" t="n"/>
+      <c r="C31" s="28" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="B33" s="11" t="inlineStr">
@@ -1662,11 +2034,11 @@
           <t>Open Output Folder</t>
         </is>
       </c>
-      <c r="C33" s="20" t="n"/>
+      <c r="C33" s="26" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="20" t="n"/>
-      <c r="C34" s="20" t="n"/>
+      <c r="B34" s="27" t="n"/>
+      <c r="C34" s="28" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Release v2.2.0 capacity routing updates
</commit_message>
<xml_diff>
--- a/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
+++ b/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
@@ -70,12 +70,12 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="007F6000"/>
+      <color rgb="00666666"/>
       <sz val="9"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="007F6000"/>
       <sz val="9"/>
     </font>
     <font>
@@ -113,12 +113,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F75B5"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="002F75B5"/>
       </patternFill>
     </fill>
   </fills>
@@ -264,21 +264,30 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -288,15 +297,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -712,7 +712,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>All</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Expansion</t>
+          <t>Baseline</t>
         </is>
       </c>
     </row>
@@ -747,13 +747,18 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lean</t>
+          <t>Expansion</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="C5" t="n">
         <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Lean</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -822,9 +827,9 @@
           <t>Deployment Steps - copy the tool, install dependencies, activate the license, and run</t>
         </is>
       </c>
-      <c r="B1" s="21" t="n"/>
-      <c r="C1" s="21" t="n"/>
-      <c r="D1" s="22" t="n"/>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="25" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -832,9 +837,9 @@
           <t>Recommended portable setup: keep Capacity_Optimizer_Control.xlsx inside 'Tooling Control Panel', then use Project_Root_Folder = '..', Input_Load_Folder = 'Data_Input', Input_Master_Folder = 'Data_Input', Output_Folder = 'output', and place 'license.json' in 'licenses\active\'. 中文说明见右侧列。</t>
         </is>
       </c>
-      <c r="B2" s="21" t="n"/>
-      <c r="C2" s="21" t="n"/>
-      <c r="D2" s="22" t="n"/>
+      <c r="B2" s="24" t="n"/>
+      <c r="C2" s="24" t="n"/>
+      <c r="D2" s="25" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1128,9 +1133,9 @@
           <t>Where to continue: open the 'Control_Panel' sheet and start with the Migration Setup section.</t>
         </is>
       </c>
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="22" t="n"/>
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1148,7 +1153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1303,90 +1308,83 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Direct_Mode: keep 'Yes' for the folder-based CSV workflow.</t>
+          <t>Verbose: prints solver detail in the command window.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Verbose: prints solver detail in the command window.</t>
+          <t>Skip_Validation_Errors: only use 'Yes' when you intentionally want a forced run.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Skip_Validation_Errors: only use 'Yes' when you intentionally want a forced run.</t>
-        </is>
-      </c>
+      <c r="A25" s="10" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr"/>
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>LICENSE</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>LICENSE</t>
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>license.json: recommended location is licenses\active\license.json; the legacy project-root path is also supported.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>license.json: recommended location is licenses\active\license.json; the legacy project-root path is also supported.</t>
+          <t>Trial / unbound license: no machine fingerprint required; RSCP can issue it directly.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>Trial / unbound license: no machine fingerprint required; RSCP can issue it directly.</t>
+          <t>runtime\get_machine_fingerprint.bat: creates a timestamped fingerprint file under licenses\requests\ for RSCP to issue a machine-locked license.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>runtime\get_machine_fingerprint.bat: creates a timestamped fingerprint file under licenses\requests\ for RSCP to issue a machine-locked license.</t>
+          <t>Run_Info: each output workbook records license status, license ID, customer, expiry date, and binding mode.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>Run_Info: each output workbook records license status, license ID, customer, expiry date, and binding mode.</t>
-        </is>
-      </c>
+      <c r="A31" s="10" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr"/>
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>RESULT WORKBOOK CONTENT</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>RESULT WORKBOOK CONTENT</t>
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard, Monthly_Trend, Bottleneck, WC_Heatmap, Product_Risk</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Dashboard, Monthly_Trend, Bottleneck, WC_Heatmap, Product_Risk</t>
+          <t>Allocation_Detail, Planner_Result_Summary</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Allocation_Detail, Allocation_Summary, Outsource_Summary, Unmet_Summary, WC_Load_Pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Binary_Feasibility, Validation_Issues, Run_Info</t>
+          <t>Validation_Issues, Run_Info</t>
         </is>
       </c>
     </row>
@@ -1415,6 +1413,8 @@
           <t>Current License</t>
         </is>
       </c>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="25" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1422,6 +1422,8 @@
           <t>This sheet shows the currently detected license for this tool copy. Values refresh when the workbook is generated and again when the optimizer can save updates back to this file.</t>
         </is>
       </c>
+      <c r="B2" s="24" t="n"/>
+      <c r="C2" s="25" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1441,204 +1443,204 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>License_Status</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Valid</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>Current validation status of the active license</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>License_Name</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>LIC-DEV-2026-0001</t>
         </is>
       </c>
-      <c r="C6" s="25" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>Current license ID / license name</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>License_Mode</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Internal / Machine Locked</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>Friendly label such as Trial / Unbound or Commercial / Machine Locked</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>License_Type</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>internal</t>
         </is>
       </c>
-      <c r="C8" s="25" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>License type from license.json</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Binding_Mode</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>machine_locked</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>Whether the license is unbound or machine locked</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Licensed_To</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>RSCP</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Customer name recorded in the license</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Issue_Date</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>License issue date</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Expiry_Date</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>2027-12-31</t>
         </is>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>License expiry date</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Machine_Name</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>HYC</t>
         </is>
       </c>
-      <c r="C13" s="25" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>Licensed machine label when applicable</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>License_File_Path</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>C:\Users\super\capacity_optimizer\licenses\active\license.json</t>
         </is>
       </c>
-      <c r="C14" s="25" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>Detected license.json location</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Local development license</t>
         </is>
       </c>
-      <c r="C15" s="25" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>Note stored inside the license file</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>License validated successfully.</t>
         </is>
       </c>
-      <c r="C16" s="25" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>Last license inspection message</t>
         </is>
@@ -1659,7 +1661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1685,13 +1687,13 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Migration Setup - update these cells first after copying the tool to another computer</t>
         </is>
       </c>
-      <c r="B2" s="21" t="n"/>
-      <c r="C2" s="22" t="n"/>
+      <c r="B2" s="24" t="n"/>
+      <c r="C2" s="25" t="n"/>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -1699,72 +1701,72 @@
           <t>Recommended portable setup: keep Project_Root_Folder = '..', Input folders = 'Data_Input', Output_Folder = 'output', and place 'license.json' in 'licenses\active\'. See 'Deployment_Steps' for the full setup checklist.</t>
         </is>
       </c>
-      <c r="B3" s="21" t="n"/>
-      <c r="C3" s="22" t="n"/>
+      <c r="B3" s="24" t="n"/>
+      <c r="C3" s="25" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Project_Root_Folder</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>..</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>Project root folder; '..' means one level above this workbook</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Input_Load_Folder</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Data_Input</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Planner folder name or full path</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Input_Master_Folder</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Data_Input</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>Master-data folder name or full path</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Output_Folder</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>output</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Result folder name or full path</t>
         </is>
@@ -1776,277 +1778,260 @@
           <t>Run Settings</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="22" t="n"/>
+      <c r="B8" s="24" t="n"/>
+      <c r="C8" s="25" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Output_FileName</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>capacity_result.xlsx</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Base name for result workbooks</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Scenario_Name</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Planner Scenario value; type manually if your data folder changes</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Start_Year</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>First planning year</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Start_Month_Num</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>First planning month number (1-12)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Start_Month</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>Optional legacy field; Python derives this from year/month first</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Horizon_Months</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>Number of monthly buckets</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Run_Mode</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>ModeA, ModeB, or Both</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Direct_Mode</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>Use direct folder-based CSV/Excel inputs</t>
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Verbose</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>Print solver detail in the command window</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Verbose</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Skip_Validation_Errors</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>Print solver detail in the command window</t>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>Run even when validation finds errors</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Skip_Validation_Errors</t>
-        </is>
-      </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>Run even when validation finds errors</t>
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Run_Timestamp</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr"/>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Filled by Python at runtime</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>Run_Timestamp</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr"/>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>Filled by Python at runtime</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr"/>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr"/>
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>Free text</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Run command</t>
         </is>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>python -m app.main --input-template "Tooling Control Panel/Capacity_Optimizer_Control.xlsx"</t>
         </is>
       </c>
     </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Quick actions</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Setup Dependencies</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="n"/>
+    </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Quick actions</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Setup Dependencies</t>
-        </is>
-      </c>
-      <c r="C24" s="26" t="n"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="27" t="n"/>
-      <c r="C25" s="28" t="n"/>
+      <c r="B24" s="27" t="n"/>
+      <c r="C24" s="28" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Get Machine Fingerprint</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Get Machine Fingerprint</t>
-        </is>
-      </c>
-      <c r="C27" s="26" t="n"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="27" t="n"/>
-      <c r="C28" s="28" t="n"/>
+      <c r="B27" s="27" t="n"/>
+      <c r="C27" s="28" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Run Optimizer</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>Run Optimizer</t>
-        </is>
-      </c>
-      <c r="C30" s="26" t="n"/>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="27" t="n"/>
-      <c r="C31" s="28" t="n"/>
+      <c r="B30" s="27" t="n"/>
+      <c r="C30" s="28" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Open Output Folder</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>Open Output Folder</t>
-        </is>
-      </c>
-      <c r="C33" s="26" t="n"/>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="27" t="n"/>
-      <c r="C34" s="28" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="B33" s="27" t="n"/>
+      <c r="C33" s="28" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>Button note</t>
         </is>
       </c>
-      <c r="B36" s="19" t="inlineStr">
+      <c r="B35" s="22" t="inlineStr">
         <is>
           <t>On a new computer, click Setup Dependencies first. If RSCP gave you a trial/unbound license, place license.json in licenses\active and continue. Otherwise click Get Machine Fingerprint, send the generated file from licenses\requests to RSCP, place the returned license.json in licenses\active, save the workbook (Ctrl+S), and click Run Optimizer.</t>
         </is>
@@ -2054,15 +2039,15 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B33:C34"/>
     <mergeCell ref="A8:C8"/>
+    <mergeCell ref="B29:C30"/>
+    <mergeCell ref="B26:C27"/>
+    <mergeCell ref="B23:C24"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="B24:C25"/>
-    <mergeCell ref="B30:C31"/>
-    <mergeCell ref="B27:C28"/>
+    <mergeCell ref="B32:C33"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$A$2:$A$4</formula1>
     </dataValidation>
@@ -2070,9 +2055,6 @@
       <formula1>=Lists!$B$2:$B$3</formula1>
     </dataValidation>
     <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$B$2:$B$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$B$2:$B$3</formula1>
     </dataValidation>
     <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2083,10 +2065,10 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Release v2.2.1 setup time capacity reporting
</commit_message>
<xml_diff>
--- a/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
+++ b/Tooling Control Panel/Capacity_Optimizer_Control.xlsx
@@ -732,7 +732,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>10 case</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Expansion</t>
+          <t>50 case</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Lean</t>
+          <t>90 case</t>
         </is>
       </c>
     </row>
@@ -1413,8 +1413,6 @@
           <t>Current License</t>
         </is>
       </c>
-      <c r="B1" s="24" t="n"/>
-      <c r="C1" s="25" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1422,8 +1420,6 @@
           <t>This sheet shows the currently detected license for this tool copy. Values refresh when the workbook is generated and again when the optimizer can save updates back to this file.</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n"/>
-      <c r="C2" s="25" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1603,7 +1599,7 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>C:\Users\super\capacity_optimizer\licenses\active\license.json</t>
+          <t>D:\RSCP_Dupont\Dupont_Capacity_Oprimizer\Capacity_Optimizer_Tools\licenses\active\license.json</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">

</xml_diff>